<commit_message>
changes suggested by amruta
</commit_message>
<xml_diff>
--- a/content/knowledge_bay_content_local.xlsx
+++ b/content/knowledge_bay_content_local.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/e131770/Desktop/team_projects/Virtual-Tourer/ai-india-summit-mc/content/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{388424E9-BCEF-8F41-9BC0-B7EAFCB36B82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3C5068C-359D-E141-9670-4295CA03F038}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="34560" windowHeight="21600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="34560" windowHeight="21600" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LandingPage" sheetId="1" r:id="rId1"/>
@@ -2531,9 +2531,6 @@
     <t>images/LoG.jpg</t>
   </si>
   <si>
-    <t>AI Garage leverages and applies Artificial Intelligence at scale within Mastercard and its associated business partners, providing a foundational, competitive advantage for the future.</t>
-  </si>
-  <si>
     <t>images/jailbreak.jpeg</t>
   </si>
   <si>
@@ -2691,6 +2688,9 @@
   </si>
   <si>
     <t>Welcome to the Knowledge Bay</t>
+  </si>
+  <si>
+    <t>AI Garage is a power house for different verticals that come together to strengthen Mastercard ecosystem</t>
   </si>
 </sst>
 </file>
@@ -3356,7 +3356,7 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="D2" t="s">
         <v>5</v>
@@ -4039,7 +4039,7 @@
         <v>659</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>660</v>
@@ -4114,7 +4114,7 @@
         <v>794</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="G10">
         <v>2025</v>
@@ -4183,7 +4183,7 @@
         <v>798</v>
       </c>
       <c r="E2" s="24" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="F2" s="25" t="s">
         <v>182</v>
@@ -4203,7 +4203,7 @@
         <v>185</v>
       </c>
       <c r="E3" s="24" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="F3" s="25" t="s">
         <v>186</v>
@@ -4223,7 +4223,7 @@
         <v>803</v>
       </c>
       <c r="E4" s="24" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="F4" s="25" t="s">
         <v>187</v>
@@ -4243,7 +4243,7 @@
         <v>190</v>
       </c>
       <c r="E5" s="24" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="F5" s="25" t="s">
         <v>191</v>
@@ -4263,7 +4263,7 @@
         <v>194</v>
       </c>
       <c r="E6" s="24" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="F6" s="25" t="s">
         <v>195</v>
@@ -4283,7 +4283,7 @@
         <v>806</v>
       </c>
       <c r="E7" s="29" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="F7" s="25" t="s">
         <v>807</v>
@@ -4303,7 +4303,7 @@
         <v>810</v>
       </c>
       <c r="E8" s="29" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="F8" s="25" t="s">
         <v>811</v>
@@ -4323,10 +4323,10 @@
         <v>815</v>
       </c>
       <c r="E9" s="29" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="F9" s="25" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
     </row>
   </sheetData>
@@ -4906,7 +4906,7 @@
       </c>
       <c r="G15" s="10"/>
       <c r="H15" s="10" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="I15" s="10" t="s">
         <v>260</v>
@@ -4943,7 +4943,7 @@
       </c>
       <c r="G16" s="11"/>
       <c r="H16" s="10" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="I16" s="11" t="s">
         <v>263</v>
@@ -5887,7 +5887,7 @@
         <v>243</v>
       </c>
       <c r="B42" s="10" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="C42" s="10" t="s">
         <v>148</v>
@@ -5924,7 +5924,7 @@
         <v>243</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="C43" s="10" t="s">
         <v>148</v>
@@ -6051,7 +6051,7 @@
       </c>
       <c r="G46" s="10"/>
       <c r="H46" s="10" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="I46" s="10" t="s">
         <v>363</v>
@@ -6457,13 +6457,13 @@
         <v>330</v>
       </c>
       <c r="I57" s="30" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="J57" s="10" t="s">
         <v>214</v>
       </c>
       <c r="K57" s="31" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="L57" s="10"/>
       <c r="M57" s="10">
@@ -6475,32 +6475,32 @@
         <v>392</v>
       </c>
       <c r="B58" s="32" t="s">
+        <v>841</v>
+      </c>
+      <c r="C58" s="32" t="s">
         <v>842</v>
       </c>
-      <c r="C58" s="32" t="s">
+      <c r="D58" s="32" t="s">
         <v>843</v>
       </c>
-      <c r="D58" s="32" t="s">
+      <c r="E58" s="22" t="s">
         <v>844</v>
       </c>
-      <c r="E58" s="22" t="s">
+      <c r="F58" s="13" t="s">
         <v>845</v>
-      </c>
-      <c r="F58" s="13" t="s">
-        <v>846</v>
       </c>
       <c r="G58" s="10"/>
       <c r="H58" s="10" t="s">
         <v>333</v>
       </c>
       <c r="I58" s="30" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="J58" s="10" t="s">
         <v>228</v>
       </c>
       <c r="K58" s="31" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="L58" s="10"/>
       <c r="M58" s="10">
@@ -6512,7 +6512,7 @@
         <v>486</v>
       </c>
       <c r="B59" s="32" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="C59" s="32" t="s">
         <v>148</v>
@@ -6524,20 +6524,20 @@
         <v>733</v>
       </c>
       <c r="F59" s="13" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="G59" s="10"/>
       <c r="H59" s="10" t="s">
         <v>337</v>
       </c>
       <c r="I59" s="30" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="J59" s="10" t="s">
         <v>214</v>
       </c>
       <c r="K59" s="31" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="L59" s="10"/>
       <c r="M59" s="10">
@@ -6549,16 +6549,16 @@
         <v>236</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="C60" s="32" t="s">
         <v>148</v>
       </c>
       <c r="D60" s="4" t="s">
+        <v>853</v>
+      </c>
+      <c r="E60" s="4" t="s">
         <v>854</v>
-      </c>
-      <c r="E60" s="4" t="s">
-        <v>855</v>
       </c>
       <c r="F60" s="13" t="s">
         <v>499</v>
@@ -6568,13 +6568,13 @@
         <v>341</v>
       </c>
       <c r="I60" s="30" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="J60" s="10" t="s">
         <v>252</v>
       </c>
       <c r="K60" s="31" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="L60" s="10"/>
       <c r="M60" s="10">
@@ -6586,32 +6586,32 @@
         <v>432</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="C61" s="32" t="s">
         <v>148</v>
       </c>
       <c r="D61" s="4" t="s">
+        <v>858</v>
+      </c>
+      <c r="E61" s="4" t="s">
         <v>859</v>
       </c>
-      <c r="E61" s="4" t="s">
+      <c r="F61" s="13" t="s">
         <v>860</v>
-      </c>
-      <c r="F61" s="13" t="s">
-        <v>861</v>
       </c>
       <c r="G61" s="10"/>
       <c r="H61" s="10" t="s">
         <v>344</v>
       </c>
       <c r="I61" s="30" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="J61" s="10" t="s">
         <v>261</v>
       </c>
       <c r="K61" s="31" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="L61" s="10"/>
       <c r="M61" s="10">
@@ -7616,7 +7616,7 @@
         <v>514</v>
       </c>
       <c r="B89" s="32" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="C89" s="8" t="s">
         <v>148</v>
@@ -7651,7 +7651,7 @@
         <v>243</v>
       </c>
       <c r="B90" s="16" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="C90" s="8" t="s">
         <v>148</v>
@@ -7721,7 +7721,7 @@
         <v>243</v>
       </c>
       <c r="B92" s="16" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="C92" s="8" t="s">
         <v>148</v>
@@ -7771,7 +7771,7 @@
         <v>754</v>
       </c>
       <c r="H93" s="10" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="I93" s="1" t="s">
         <v>755</v>
@@ -7806,7 +7806,7 @@
         <v>757</v>
       </c>
       <c r="H94" s="10" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="I94" s="23" t="s">
         <v>758</v>
@@ -7826,19 +7826,19 @@
         <v>739</v>
       </c>
       <c r="B95" s="34" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="C95" s="8" t="s">
         <v>148</v>
       </c>
       <c r="D95" s="21" t="s">
+        <v>874</v>
+      </c>
+      <c r="E95" s="21" t="s">
         <v>875</v>
       </c>
-      <c r="E95" s="21" t="s">
+      <c r="F95" s="8" t="s">
         <v>876</v>
-      </c>
-      <c r="F95" s="8" t="s">
-        <v>877</v>
       </c>
       <c r="H95" s="10"/>
       <c r="I95" s="8" t="s">
@@ -7865,13 +7865,13 @@
         <v>148</v>
       </c>
       <c r="D96" s="4" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="E96" s="4" t="s">
         <v>742</v>
       </c>
       <c r="F96" s="8" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="I96" s="8" t="s">
         <v>730</v>
@@ -7954,7 +7954,7 @@
         <v>816</v>
       </c>
       <c r="C2" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="D2" t="s">
         <v>16</v>
@@ -7971,7 +7971,7 @@
         <v>19</v>
       </c>
       <c r="C3" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="D3" t="s">
         <v>20</v>
@@ -7988,7 +7988,7 @@
         <v>817</v>
       </c>
       <c r="C4" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="D4" t="s">
         <v>24</v>
@@ -8094,7 +8094,7 @@
         <v>28</v>
       </c>
       <c r="B3" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="D3" t="s">
         <v>34</v>
@@ -8383,7 +8383,7 @@
         <v>80</v>
       </c>
       <c r="B4" t="s">
-        <v>827</v>
+        <v>880</v>
       </c>
       <c r="D4" t="s">
         <v>81</v>
@@ -8515,7 +8515,7 @@
         <v>97</v>
       </c>
       <c r="C4" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="D4" t="s">
         <v>98</v>

</xml_diff>